<commit_message>
Separate cold store and grocery counters
</commit_message>
<xml_diff>
--- a/outputs/oneroot-essentials-register/OneRoot_Essentials_Operations_Register.xlsx
+++ b/outputs/oneroot-essentials-register/OneRoot_Essentials_Operations_Register.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R0eaf963826de4724"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expenses" sheetId="2" r:id="R39319178ab6f4757"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget_Planner" sheetId="3" r:id="Rd071e9fc7388474e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_Sales" sheetId="4" r:id="Ra9f88615a20a4bae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apartments" sheetId="5" r:id="Rb33e04d96ca742a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petty_Cash" sheetId="6" r:id="Rc4e788c15d0f47b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petty_Cash_Budget" sheetId="7" r:id="R5367aa11eda144ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary_Register" sheetId="8" r:id="Rc52e20ce8d684819"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier_Ledger" sheetId="9" r:id="Rd62c136bdfaa48a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recurring_Controls" sheetId="10" r:id="Rba43ffcba59043c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maintenance_Log" sheetId="11" r:id="R688096d8c97c4dd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="12" r:id="Rcfdc9fd8ac9345c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ref8673abdb4c4a02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expenses" sheetId="2" r:id="R11350bdeaf954bb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget_Planner" sheetId="3" r:id="R7775ad41846642e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_Sales" sheetId="4" r:id="R88fc82c5e0dc4b42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apartments" sheetId="5" r:id="Rcbce5c9879c84784"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petty_Cash" sheetId="6" r:id="R4723797c3b734044"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petty_Cash_Budget" sheetId="7" r:id="R3b50add91f7342a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary_Register" sheetId="8" r:id="R263f4c928ef74fb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier_Ledger" sheetId="9" r:id="R6ed3abaeb06f4daf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recurring_Controls" sheetId="10" r:id="R09900fb5ba874d5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maintenance_Log" sheetId="11" r:id="R90907046d0eb430d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="12" r:id="R8496fd2b9fe446d8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -558,9 +558,9 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="171.3300018310547" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="170.22000122070312" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="7.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="27.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="29.110000610351562" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
@@ -640,7 +640,7 @@
       </x:c>
       <x:c r="C6" s="33"/>
       <x:c r="D6" s="32" t="str">
-        <x:v>OneRoot Cold Store &amp; Groceries</x:v>
+        <x:v>OneRoot Cold Store &amp; Kitchen</x:v>
       </x:c>
       <x:c r="E6" s="33" t="str"/>
       <x:c r="F6" s="33" t="str"/>
@@ -657,7 +657,7 @@
       </x:c>
       <x:c r="C7" s="33"/>
       <x:c r="D7" s="32" t="str">
-        <x:v>OneRoot Laundry Services</x:v>
+        <x:v>OneRoot Groceries &amp; More</x:v>
       </x:c>
       <x:c r="E7" s="33" t="str"/>
       <x:c r="F7" s="33" t="str"/>
@@ -674,7 +674,7 @@
       </x:c>
       <x:c r="C8" s="33"/>
       <x:c r="D8" s="32" t="str">
-        <x:v>OneRoot Mobile Money Services</x:v>
+        <x:v>OneRoot Laundry Services</x:v>
       </x:c>
       <x:c r="E8" s="33" t="str"/>
       <x:c r="F8" s="33" t="str"/>
@@ -691,7 +691,7 @@
       </x:c>
       <x:c r="C9" s="33"/>
       <x:c r="D9" s="32" t="str">
-        <x:v>OneRoot Rentals &amp; Apartments</x:v>
+        <x:v>OneRoot Mobile Money Services</x:v>
       </x:c>
       <x:c r="E9" s="33" t="str"/>
       <x:c r="F9" s="33" t="str"/>
@@ -708,7 +708,7 @@
       </x:c>
       <x:c r="C10" s="33"/>
       <x:c r="D10" s="32" t="str">
-        <x:v>OneRoot Fresh Foods &amp; Drinks</x:v>
+        <x:v>OneRoot Rentals &amp; Apartments</x:v>
       </x:c>
       <x:c r="E10" s="33" t="str"/>
       <x:c r="F10" s="33" t="str"/>
@@ -725,7 +725,7 @@
       </x:c>
       <x:c r="C11" s="33"/>
       <x:c r="D11" s="32" t="str">
-        <x:v>OneRoot Kitchen</x:v>
+        <x:v>OneRoot Fresh Foods &amp; Drinks</x:v>
       </x:c>
       <x:c r="E11" s="33" t="str"/>
       <x:c r="F11" s="33" t="str"/>
@@ -741,13 +741,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C12" s="33"/>
-      <x:c r="D12" s="34" t="str">
-        <x:v>OneRoot Shared Operations</x:v>
-      </x:c>
-      <x:c r="E12" s="35" t="str"/>
-      <x:c r="F12" s="35" t="str"/>
-      <x:c r="G12" s="35" t="str"/>
-      <x:c r="H12" s="12" t="str"/>
+      <x:c r="D12" s="32" t="str">
+        <x:v>OneRoot Kitchen</x:v>
+      </x:c>
+      <x:c r="E12" s="33" t="str"/>
+      <x:c r="F12" s="33" t="str"/>
+      <x:c r="G12" s="33" t="str"/>
+      <x:c r="H12" s="10" t="str"/>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="19" t="str">
@@ -758,11 +758,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C13" s="33"/>
-      <x:c r="D13" s="33"/>
-      <x:c r="E13" s="33"/>
-      <x:c r="F13" s="33"/>
-      <x:c r="G13" s="33"/>
-      <x:c r="H13" s="10"/>
+      <x:c r="D13" s="34" t="str">
+        <x:v>OneRoot Shared Operations</x:v>
+      </x:c>
+      <x:c r="E13" s="35" t="str"/>
+      <x:c r="F13" s="35" t="str"/>
+      <x:c r="G13" s="35" t="str"/>
+      <x:c r="H13" s="12" t="str"/>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="19" t="str">
@@ -1005,21 +1007,21 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="6" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="10.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="10.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="11" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="8.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="7.889999866485596" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="15.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="5.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="9.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="4.78000020980835" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="5.21999979019165" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="6.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="11.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="11.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="8.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="8.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="11.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="6.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="9.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="5.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="5.440000057220459" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -3766,7 +3768,7 @@
       <x:formula1>'Lists'!$J$2:$J$5</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C2:C300">
-      <x:formula1>'Lists'!$A$2:$A$9</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D2:D300">
       <x:formula1>'Lists'!$B$2:$B$46</x:formula1>
@@ -3789,18 +3791,18 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="9.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="9.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="5.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="5.21999979019165" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="7.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="16.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="13.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="14.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="4.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="9.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="9.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="6.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="5.440000057220459" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="7.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="15.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="5.110000133514404" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -5638,7 +5640,7 @@
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B2:B300">
-      <x:formula1>'Lists'!$A$2:$A$9</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F2:F300">
       <x:formula1>'Lists'!$L$2:$L$5</x:formula1>
@@ -5657,18 +5659,18 @@
   <x:cols>
     <x:col min="1" max="1" width="27.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="23.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="13.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="11.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="15.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="9.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="13.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="14.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="16.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="16.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="16.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="10.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="9.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="15.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="17.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="10.779999732971191" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="11.329999923706055" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -5768,7 +5770,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>OneRoot Cold Store &amp; Groceries</x:v>
+        <x:v>OneRoot Cold Store &amp; Kitchen</x:v>
       </x:c>
       <x:c r="B3" t="str">
         <x:v>Equipment Repairs</x:v>
@@ -5815,7 +5817,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>OneRoot Laundry Services</x:v>
+        <x:v>OneRoot Groceries &amp; More</x:v>
       </x:c>
       <x:c r="B4" t="str">
         <x:v>Fuel &amp; Delivery</x:v>
@@ -5859,7 +5861,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>OneRoot Mobile Money Services</x:v>
+        <x:v>OneRoot Laundry Services</x:v>
       </x:c>
       <x:c r="B5" t="str">
         <x:v>Tools &amp; Consumables</x:v>
@@ -5897,7 +5899,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>OneRoot Rentals &amp; Apartments</x:v>
+        <x:v>OneRoot Mobile Money Services</x:v>
       </x:c>
       <x:c r="B6" t="str">
         <x:v>Site Labour</x:v>
@@ -5917,7 +5919,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>OneRoot Fresh Foods &amp; Drinks</x:v>
+        <x:v>OneRoot Rentals &amp; Apartments</x:v>
       </x:c>
       <x:c r="B7" t="str">
         <x:v>Utilities</x:v>
@@ -5934,7 +5936,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>OneRoot Kitchen</x:v>
+        <x:v>OneRoot Fresh Foods &amp; Drinks</x:v>
       </x:c>
       <x:c r="B8" t="str">
         <x:v>Marketing &amp; Promotion</x:v>
@@ -5945,7 +5947,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>OneRoot Shared Operations</x:v>
+        <x:v>OneRoot Kitchen</x:v>
       </x:c>
       <x:c r="B9" t="str">
         <x:v>Professional Services</x:v>
@@ -5955,6 +5957,9 @@
       </x:c>
     </x:row>
     <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>OneRoot Shared Operations</x:v>
+      </x:c>
       <x:c r="B10" t="str">
         <x:v>Rent &amp; Space</x:v>
       </x:c>
@@ -6178,15 +6183,15 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="3.890000104904175" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="11.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="10.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="8.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="11.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="11" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="4.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="4.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="9.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="11.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="11.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="5.110000133514404" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -9510,7 +9515,7 @@
   </x:sheetData>
   <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="B2:B300">
-      <x:formula1>'Lists'!$A$2:$A$9</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D2:D300">
       <x:formula1>'Lists'!$B$2:$B$46</x:formula1>
@@ -9530,13 +9535,13 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="10.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="15.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="11.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="4.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="11.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="5.110000133514404" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -13153,7 +13158,7 @@
   </x:sheetData>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="B2:B300">
-      <x:formula1>'Lists'!$A$2:$A$9</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C2:C300">
       <x:formula1>'Lists'!$B$2:$B$46</x:formula1>
@@ -13167,10 +13172,10 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="3.890000104904175" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="17.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="4.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="4.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="5.110000133514404" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -14386,7 +14391,7 @@
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="B2:B300">
-      <x:formula1>'Lists'!$A$2:$A$9</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14397,43 +14402,43 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="4.21999979019165" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="5.21999979019165" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="5.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="10.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="5" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="6.559999942779541" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="7.889999866485596" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="8.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="15.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="12.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="12.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="11.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="10.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="14.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="16.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="11.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="12.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="11.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="15.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="12.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="26" max="26" width="10" hidden="0" customWidth="1"/>
-    <x:col min="27" max="27" width="12" hidden="0" customWidth="1"/>
-    <x:col min="28" max="28" width="13.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="29" max="29" width="15.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="30" max="30" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="31" max="31" width="13.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="32" max="32" width="11.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="33" max="33" width="14.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="34" max="34" width="13.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="35" max="35" width="4.78000020980835" hidden="0" customWidth="1"/>
-    <x:col min="36" max="36" width="15.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="37" max="37" width="18.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="10.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="4.440000057220459" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="5.440000057220459" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="5.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="5.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="6.889999866485596" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="8.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="9" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="16.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="12.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="13" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="12.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="11.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="11.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="11.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="15.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="17.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="12.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="12.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="12.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="15.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="13.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="10.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="12.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="14.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="16.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="11.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="14.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="12.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="33" max="33" width="15.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="14.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="35" max="35" width="5.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="36" max="36" width="16.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="37" max="37" width="19.440000534057617" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -23844,15 +23849,15 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="3.890000104904175" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="12.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="10.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="10.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="11.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="11" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="4.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="4.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="11.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="11.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="11.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="5.110000133514404" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -26282,7 +26287,7 @@
       <x:formula1>'Lists'!$F$2:$F$7</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C2:C300">
-      <x:formula1>'Lists'!$A$2:$A$9</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D2:D300">
       <x:formula1>'Lists'!$B$2:$B$46</x:formula1>
@@ -26299,10 +26304,10 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="4.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="17.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="5.110000133514404" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -27518,7 +27523,7 @@
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="B2:B300">
-      <x:formula1>'Lists'!$A$2:$A$9</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -27529,27 +27534,27 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="8.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="8.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="15.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16.219999313354492" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="14.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="14.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="7.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="10.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="13" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="14.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="5.21999979019165" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="4.78000020980835" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="8.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="6.440000057220459" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="8" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="8.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="15" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="9.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="9.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="15.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="15.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="7.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="11.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="13.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="15.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="5.440000057220459" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="5.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="8.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="6.889999866485596" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="8.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="8.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="15.890000343322754" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -34796,7 +34801,7 @@
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B2:B300">
-      <x:formula1>'Lists'!$A$2:$A$9</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="E2:E300">
       <x:formula1>'Lists'!$O$2:$O$6</x:formula1>
@@ -34813,20 +34818,20 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="9.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="6.559999942779541" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="10.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="13.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="14.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="14.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="7.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="10.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="13" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="20.559999465942383" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="5.21999979019165" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="4.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="10.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="6.889999866485596" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="15.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="7.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="11.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="13.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="21.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="5.440000057220459" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="5.110000133514404" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -39062,7 +39067,7 @@
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B2:B300">
-      <x:formula1>'Lists'!$A$2:$A$9</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D2:D300">
       <x:formula1>'Lists'!$B$2:$B$46</x:formula1>

</xml_diff>

<commit_message>
Add phone accessories and construction areas
</commit_message>
<xml_diff>
--- a/outputs/oneroot-essentials-register/OneRoot_Essentials_Operations_Register.xlsx
+++ b/outputs/oneroot-essentials-register/OneRoot_Essentials_Operations_Register.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ref8673abdb4c4a02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expenses" sheetId="2" r:id="R11350bdeaf954bb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget_Planner" sheetId="3" r:id="R7775ad41846642e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_Sales" sheetId="4" r:id="R88fc82c5e0dc4b42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apartments" sheetId="5" r:id="Rcbce5c9879c84784"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petty_Cash" sheetId="6" r:id="R4723797c3b734044"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petty_Cash_Budget" sheetId="7" r:id="R3b50add91f7342a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary_Register" sheetId="8" r:id="R263f4c928ef74fb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier_Ledger" sheetId="9" r:id="R6ed3abaeb06f4daf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recurring_Controls" sheetId="10" r:id="R09900fb5ba874d5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maintenance_Log" sheetId="11" r:id="R90907046d0eb430d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="12" r:id="R8496fd2b9fe446d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R832c09e11fb04345"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expenses" sheetId="2" r:id="Rcb3550c1107c42ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget_Planner" sheetId="3" r:id="Re1efe6fbf93c4450"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_Sales" sheetId="4" r:id="Rb0256c52e7bb4a26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apartments" sheetId="5" r:id="R2a7c95e3600d4d2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petty_Cash" sheetId="6" r:id="R28a7e4652f7a4d64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petty_Cash_Budget" sheetId="7" r:id="R3b57f94664444aad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary_Register" sheetId="8" r:id="R823e39f90a464618"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier_Ledger" sheetId="9" r:id="R833927820b814e21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recurring_Controls" sheetId="10" r:id="R99733e54896b446e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maintenance_Log" sheetId="11" r:id="Rf87787594e584768"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="12" r:id="Rc6a9598bd1924d2c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -560,7 +560,7 @@
   <x:cols>
     <x:col min="1" max="1" width="170.22000122070312" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="7.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="29.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="35.779998779296875" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
@@ -674,7 +674,7 @@
       </x:c>
       <x:c r="C8" s="33"/>
       <x:c r="D8" s="32" t="str">
-        <x:v>OneRoot Laundry Services</x:v>
+        <x:v>OneRoot Phone Accessories &amp; Charging</x:v>
       </x:c>
       <x:c r="E8" s="33" t="str"/>
       <x:c r="F8" s="33" t="str"/>
@@ -691,7 +691,7 @@
       </x:c>
       <x:c r="C9" s="33"/>
       <x:c r="D9" s="32" t="str">
-        <x:v>OneRoot Mobile Money Services</x:v>
+        <x:v>OneRoot Construction Consumables Express</x:v>
       </x:c>
       <x:c r="E9" s="33" t="str"/>
       <x:c r="F9" s="33" t="str"/>
@@ -708,7 +708,7 @@
       </x:c>
       <x:c r="C10" s="33"/>
       <x:c r="D10" s="32" t="str">
-        <x:v>OneRoot Rentals &amp; Apartments</x:v>
+        <x:v>OneRoot Laundry Services</x:v>
       </x:c>
       <x:c r="E10" s="33" t="str"/>
       <x:c r="F10" s="33" t="str"/>
@@ -725,7 +725,7 @@
       </x:c>
       <x:c r="C11" s="33"/>
       <x:c r="D11" s="32" t="str">
-        <x:v>OneRoot Fresh Foods &amp; Drinks</x:v>
+        <x:v>OneRoot Mobile Money Services</x:v>
       </x:c>
       <x:c r="E11" s="33" t="str"/>
       <x:c r="F11" s="33" t="str"/>
@@ -742,7 +742,7 @@
       </x:c>
       <x:c r="C12" s="33"/>
       <x:c r="D12" s="32" t="str">
-        <x:v>OneRoot Kitchen</x:v>
+        <x:v>OneRoot Rentals &amp; Apartments</x:v>
       </x:c>
       <x:c r="E12" s="33" t="str"/>
       <x:c r="F12" s="33" t="str"/>
@@ -758,13 +758,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C13" s="33"/>
-      <x:c r="D13" s="34" t="str">
-        <x:v>OneRoot Shared Operations</x:v>
-      </x:c>
-      <x:c r="E13" s="35" t="str"/>
-      <x:c r="F13" s="35" t="str"/>
-      <x:c r="G13" s="35" t="str"/>
-      <x:c r="H13" s="12" t="str"/>
+      <x:c r="D13" s="32" t="str">
+        <x:v>OneRoot Fresh Foods &amp; Drinks</x:v>
+      </x:c>
+      <x:c r="E13" s="33" t="str"/>
+      <x:c r="F13" s="33" t="str"/>
+      <x:c r="G13" s="33" t="str"/>
+      <x:c r="H13" s="10" t="str"/>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="19" t="str">
@@ -775,11 +775,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C14" s="33"/>
-      <x:c r="D14" s="33"/>
-      <x:c r="E14" s="33"/>
-      <x:c r="F14" s="33"/>
-      <x:c r="G14" s="33"/>
-      <x:c r="H14" s="10"/>
+      <x:c r="D14" s="32" t="str">
+        <x:v>OneRoot Kitchen</x:v>
+      </x:c>
+      <x:c r="E14" s="33" t="str"/>
+      <x:c r="F14" s="33" t="str"/>
+      <x:c r="G14" s="33" t="str"/>
+      <x:c r="H14" s="10" t="str"/>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="19" t="str">
@@ -790,11 +792,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C15" s="33"/>
-      <x:c r="D15" s="33"/>
-      <x:c r="E15" s="33"/>
-      <x:c r="F15" s="33"/>
-      <x:c r="G15" s="33"/>
-      <x:c r="H15" s="10"/>
+      <x:c r="D15" s="34" t="str">
+        <x:v>OneRoot Shared Operations</x:v>
+      </x:c>
+      <x:c r="E15" s="35" t="str"/>
+      <x:c r="F15" s="35" t="str"/>
+      <x:c r="G15" s="35" t="str"/>
+      <x:c r="H15" s="12" t="str"/>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="19" t="str">
@@ -3768,7 +3772,7 @@
       <x:formula1>'Lists'!$J$2:$J$5</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C2:C300">
-      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$12</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D2:D300">
       <x:formula1>'Lists'!$B$2:$B$46</x:formula1>
@@ -5640,7 +5644,7 @@
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B2:B300">
-      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$12</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F2:F300">
       <x:formula1>'Lists'!$L$2:$L$5</x:formula1>
@@ -5657,7 +5661,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="27.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="33.66999816894531" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="23.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="14.5600004196167" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="13.670000076293945" hidden="0" customWidth="1"/>
@@ -5861,7 +5865,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>OneRoot Laundry Services</x:v>
+        <x:v>OneRoot Phone Accessories &amp; Charging</x:v>
       </x:c>
       <x:c r="B5" t="str">
         <x:v>Tools &amp; Consumables</x:v>
@@ -5899,7 +5903,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>OneRoot Mobile Money Services</x:v>
+        <x:v>OneRoot Construction Consumables Express</x:v>
       </x:c>
       <x:c r="B6" t="str">
         <x:v>Site Labour</x:v>
@@ -5919,7 +5923,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>OneRoot Rentals &amp; Apartments</x:v>
+        <x:v>OneRoot Laundry Services</x:v>
       </x:c>
       <x:c r="B7" t="str">
         <x:v>Utilities</x:v>
@@ -5936,7 +5940,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>OneRoot Fresh Foods &amp; Drinks</x:v>
+        <x:v>OneRoot Mobile Money Services</x:v>
       </x:c>
       <x:c r="B8" t="str">
         <x:v>Marketing &amp; Promotion</x:v>
@@ -5947,7 +5951,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>OneRoot Kitchen</x:v>
+        <x:v>OneRoot Rentals &amp; Apartments</x:v>
       </x:c>
       <x:c r="B9" t="str">
         <x:v>Professional Services</x:v>
@@ -5958,7 +5962,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>OneRoot Shared Operations</x:v>
+        <x:v>OneRoot Fresh Foods &amp; Drinks</x:v>
       </x:c>
       <x:c r="B10" t="str">
         <x:v>Rent &amp; Space</x:v>
@@ -5968,6 +5972,9 @@
       </x:c>
     </x:row>
     <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>OneRoot Kitchen</x:v>
+      </x:c>
       <x:c r="B11" t="str">
         <x:v>Inventory Purchase</x:v>
       </x:c>
@@ -5976,6 +5983,9 @@
       </x:c>
     </x:row>
     <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>OneRoot Shared Operations</x:v>
+      </x:c>
       <x:c r="B12" t="str">
         <x:v>Cold Chain Utilities</x:v>
       </x:c>
@@ -9515,7 +9525,7 @@
   </x:sheetData>
   <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="B2:B300">
-      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$12</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D2:D300">
       <x:formula1>'Lists'!$B$2:$B$46</x:formula1>
@@ -13158,7 +13168,7 @@
   </x:sheetData>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="B2:B300">
-      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$12</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C2:C300">
       <x:formula1>'Lists'!$B$2:$B$46</x:formula1>
@@ -14391,7 +14401,7 @@
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="B2:B300">
-      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$12</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -26287,7 +26297,7 @@
       <x:formula1>'Lists'!$F$2:$F$7</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C2:C300">
-      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$12</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D2:D300">
       <x:formula1>'Lists'!$B$2:$B$46</x:formula1>
@@ -27523,7 +27533,7 @@
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="B2:B300">
-      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$12</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -34801,7 +34811,7 @@
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B2:B300">
-      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$12</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="E2:E300">
       <x:formula1>'Lists'!$O$2:$O$6</x:formula1>
@@ -39067,7 +39077,7 @@
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B2:B300">
-      <x:formula1>'Lists'!$A$2:$A$10</x:formula1>
+      <x:formula1>'Lists'!$A$2:$A$12</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D2:D300">
       <x:formula1>'Lists'!$B$2:$B$46</x:formula1>

</xml_diff>